<commit_message>
chore: update Import Grade Template.xlsx
</commit_message>
<xml_diff>
--- a/resources/templates/Import Grade Template.xlsx
+++ b/resources/templates/Import Grade Template.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="MasterData" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+  <si>
+    <t>เทอม</t>
+  </si>
   <si>
     <t>รหัสนิสิต</t>
   </si>
@@ -19,6 +23,15 @@
     <t>รหัสวิชา</t>
   </si>
   <si>
+    <t>ภาคต้น</t>
+  </si>
+  <si>
+    <t>ภาคปลาย</t>
+  </si>
+  <si>
+    <t>ภาคฤดูร้อน</t>
+  </si>
+  <si>
     <t>ประเภท</t>
   </si>
   <si>
@@ -26,9 +39,6 @@
   </si>
   <si>
     <t>ปี</t>
-  </si>
-  <si>
-    <t>เทอม</t>
   </si>
   <si>
     <t>01208111</t>
@@ -63,12 +73,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA4C2F4"/>
+        <bgColor rgb="FFA4C2F4"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -97,11 +113,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -119,6 +138,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -331,43 +354,80 @@
   </cols>
   <sheetData>
     <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>6.020500357E9</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="3">
+        <v>2565.0</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2">
+      <formula1>MasterData!$A$2:$A$4</formula1>
+    </dataValidation>
+  </dataValidations>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>6.020500357E9</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2">
-        <v>65.0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>